<commit_message>
v0.52 notes and roster (Omens sheet)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LZxrSwGT89pL2wX71oYkpZ
</commit_message>
<xml_diff>
--- a/daily-dungeon-characters.xlsx
+++ b/daily-dungeon-characters.xlsx
@@ -11,13 +11,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Party &amp; programs" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies (by family)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personalities" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Omens" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$F$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Party &amp; programs'!$A$1:$D$154</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Enemies (by family)'!$A$1:$E$328</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Personalities'!$A$1:$D$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Omens'!$A$1:$C$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -14394,6 +14396,621 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Omen</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Effect (all day)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line 1 text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Ordinary day: no effect (about half of all days)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Your load will be counted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Ordinary day: no effect (about half of all days)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>The deep learns your name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Ordinary day: no effect (about half of all days)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Someone walked here before.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Ordinary day: no effect (about half of all days)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Count the doors. Count again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Ordinary day: no effect (about half of all days)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>The ninth bell has not rung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Ordinary day: no effect (about half of all days)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>What is below was once above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Ordinary day: no effect (about half of all days)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>A light is left on for you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Ordinary day: no effect (about half of all days)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>The stone dreams of the sea.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Ordinary day: no effect (about half of all days)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Not every silence is empty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Ordinary day: no effect (about half of all days)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>A promise kept, far below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Data demons twice as likely</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>The wires remember.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Data demons twice as likely</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Something is counting down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Data demons twice as likely</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>A dial tone, far away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>folk</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Folklore demons twice as likely</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Old things walk early.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>folk</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Folklore demons twice as likely</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Salt on the wind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>folk</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Folklore demons twice as likely</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>The old ones stir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>heat</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Rooms heat up twice as fast</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Do not linger.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>heat</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Rooms heat up twice as fast</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>The room is listening today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>heat</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Rooms heat up twice as fast</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Short stays. Quiet feet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Searching finds half as much</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>The walls keep their secrets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Searching finds half as much</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Every seam is sealed today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Searching finds half as much</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>The stone stays shut.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Searching finds 1.6x as much</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>A door is open somewhere.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Searching finds 1.6x as much</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Something is loose in stone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Searching finds 1.6x as much</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>The seams are soft today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>talk</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Talking works 1.6x as often</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Strangers listen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>talk</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Talking works 1.6x as often</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Today, they will hear you out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>talk</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Talking works 1.6x as often</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Speak first. They are lonely.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>calm</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Rooms heat up half as fast</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>The halls are sleeping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>calm</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Rooms heat up half as fast</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Soft steps go unheard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>calm</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Rooms heat up half as fast</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Even the walls are tired.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>loot</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Loot drops 3x as often</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>The deep is generous today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>loot</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Loot drops 3x as often</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Something precious is near.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>loot</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Loot drops 3x as often</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Fortune favors the patient.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C35"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
v1.04 notes: internal changelog, aura in the creature sheet, voice guide
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ra4YzVt7KpmT8wZQpkPNW
</commit_message>
<xml_diff>
--- a/daily-dungeon-characters.xlsx
+++ b/daily-dungeon-characters.xlsx
@@ -13,6 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personalities" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Omens" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KURA aura reads" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Moon" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$F$45</definedName>
@@ -28,7 +31,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +51,9 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -90,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -108,6 +114,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -473,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -515,6 +522,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>Aura name</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -543,6 +555,11 @@
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -571,6 +588,11 @@
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>STRAY</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -599,6 +621,11 @@
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -627,6 +654,11 @@
           <t>Guards the party: blows land softer.</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -655,6 +687,11 @@
           <t>Mends the party after a fight. Steadies corrupted data.</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -683,6 +720,11 @@
           <t>At camp, keeps a copy of a COMMON item.</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -711,6 +753,11 @@
           <t>Reads the walls: now and then a search shows what a door hides.</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -739,6 +786,11 @@
           <t>At camp, merges two COMMON items into an UNCOMMON one.</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -767,6 +819,11 @@
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -795,6 +852,11 @@
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -823,6 +885,11 @@
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -851,6 +918,11 @@
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -879,6 +951,11 @@
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -911,6 +988,11 @@
           <t>alignment differs from its family</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>STATIC</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -939,6 +1021,11 @@
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -967,6 +1054,11 @@
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>HUM</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -999,6 +1091,11 @@
           <t>alignment differs from its family</t>
         </is>
       </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>HUM</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1031,6 +1128,11 @@
           <t>alignment differs from its family</t>
         </is>
       </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1059,6 +1161,11 @@
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>HUM</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1087,6 +1194,11 @@
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>HUM</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1115,6 +1227,11 @@
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>HUM</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1143,6 +1260,11 @@
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>STRAY HUM</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1171,6 +1293,11 @@
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>STRAY HUM</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1199,6 +1326,11 @@
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>STRAY HUM</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1227,6 +1359,11 @@
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>STRAY HUM</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1255,6 +1392,11 @@
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>STRAY HUM</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1283,6 +1425,11 @@
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>STRAY HUM</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1311,6 +1458,11 @@
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>STRAY HUM</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1343,6 +1495,11 @@
           <t>alignment differs from its family</t>
         </is>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>FERAL STATIC</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1371,6 +1528,11 @@
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>STRAY HUM</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1399,6 +1561,11 @@
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>STRAY HUM</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1427,6 +1594,11 @@
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>STRAY HUM</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1455,6 +1627,11 @@
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1483,6 +1660,11 @@
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1511,6 +1693,11 @@
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1539,6 +1726,11 @@
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1567,6 +1759,11 @@
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1595,6 +1792,11 @@
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1623,6 +1825,11 @@
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1651,6 +1858,11 @@
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1679,6 +1891,11 @@
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1707,6 +1924,11 @@
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1735,6 +1957,11 @@
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1780,7 +2007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D154"/>
+  <dimension ref="A1:D160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5174,6 +5401,138 @@
       <c r="D154" s="2" t="inlineStr">
         <is>
           <t>CU SITH sighs, once, like a bellows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>CU SITH</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Party member</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Remarks on a NOTICED aura</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>CU SITH sniffs at KURA's bag, very interested.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>CU SITH</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Party member</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Remarks on a LOUD aura</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>CU SITH's ears go flat at whatever KURA carries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>CU SITH</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Party member</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>KURA carries a MOON thing</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>CU SITH whines at the light in KURA's bag.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>CU SITH</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Party member</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Read with AURA (hint)</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>CU SITH stares back. Fair.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>CU SITH</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Party member</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Read with AURA (hint)</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Good dog energy. Still a hound.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>CU SITH</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Party member</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Read with AURA (hint)</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>It would like you to throw something.</t>
         </is>
       </c>
     </row>
@@ -5189,7 +5548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E328"/>
+  <dimension ref="A1:E348"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14050,6 +14409,546 @@
         </is>
       </c>
       <c r="E328" s="2" t="inlineStr">
+        <is>
+          <t>REDCAP, GAKI, BANSHEE, BARGHEST, TROLL, GHOUL, ONI, KAPPA, LAMIA, WRAITH, IMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Remarks on a NOTICED aura</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>{n}: "SIGNAL STRENGTH: MODERATE. SOURCE: YOU."</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>PING, DAEMON, CRON, NULL, PACKET, WORM, TRACER</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Remarks on a NOTICED aura</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>{n}: "YOU ARE BROADCASTING."</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>PING, DAEMON, CRON, NULL, PACKET, WORM, TRACER</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Remarks on a LOUD aura</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>{n}: "SIGNAL STRENGTH: EXTREME. TURN IT DOWN."</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>PING, DAEMON, CRON, NULL, PACKET, WORM, TRACER</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Remarks on a LOUD aura</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>{n}: "THAT IS A LOT OF NOISE FOR ONE USER."</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>PING, DAEMON, CRON, NULL, PACKET, WORM, TRACER</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>KURA carries a MOON thing</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>{n}: "UNKNOWN OBJECT IN USER INVENTORY. ORIGIN: UP."</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>PING, DAEMON, CRON, NULL, PACKET, WORM, TRACER</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>hardware</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Remarks on a NOTICED aura</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>{n}: "you're kinda loud, you know that?"</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>STATIC RAT, PAGER GHOUL, VENDOR, SCRAPPER, DEADLINK, LOOP SHADE</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>hardware</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Remarks on a NOTICED aura</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>{n}: "something on you is humming"</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>STATIC RAT, PAGER GHOUL, VENDOR, SCRAPPER, DEADLINK, LOOP SHADE</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>hardware</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Remarks on a LOUD aura</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>{n}: "what are you CARRYING. it's so loud"</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>STATIC RAT, PAGER GHOUL, VENDOR, SCRAPPER, DEADLINK, LOOP SHADE</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>hardware</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Remarks on a LOUD aura</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>{n}: "my fans spun up when you walked in"</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>STATIC RAT, PAGER GHOUL, VENDOR, SCRAPPER, DEADLINK, LOOP SHADE</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>hardware</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>KURA carries a MOON thing</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>{n}: "is that... from the sky?"</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>STATIC RAT, PAGER GHOUL, VENDOR, SCRAPPER, DEADLINK, LOOP SHADE</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Remarks on a NOTICED aura</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>{n}: "You hum, traveler. Both halves of me can hear it."</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>CHROME HOUND, WIRE WITCH, HEX DRONE, SERVER GOLEM, NEON DRYAD, COIN WRAITH, CHROME ONI, KITSUNE.EXE, PIXEL SPRITE, STATIC BANSHEE, LOOP LICH</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Remarks on a NOTICED aura</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>{n}: "Something in your bag is talking."</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>CHROME HOUND, WIRE WITCH, HEX DRONE, SERVER GOLEM, NEON DRYAD, COIN WRAITH, CHROME ONI, KITSUNE.EXE, PIXEL SPRITE, STATIC BANSHEE, LOOP LICH</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Remarks on a LOUD aura</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>{n}: "You blaze like a server room, flesh."</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>CHROME HOUND, WIRE WITCH, HEX DRONE, SERVER GOLEM, NEON DRYAD, COIN WRAITH, CHROME ONI, KITSUNE.EXE, PIXEL SPRITE, STATIC BANSHEE, LOOP LICH</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Remarks on a LOUD aura</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>{n}: "Traveler. Whatever you carry, it is screaming."</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>CHROME HOUND, WIRE WITCH, HEX DRONE, SERVER GOLEM, NEON DRYAD, COIN WRAITH, CHROME ONI, KITSUNE.EXE, PIXEL SPRITE, STATIC BANSHEE, LOOP LICH</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>KURA carries a MOON thing</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>{n}: "You carry a piece of the moon. Bold."</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>CHROME HOUND, WIRE WITCH, HEX DRONE, SERVER GOLEM, NEON DRYAD, COIN WRAITH, CHROME ONI, KITSUNE.EXE, PIXEL SPRITE, STATIC BANSHEE, LOOP LICH</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>folklore</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Remarks on a NOTICED aura</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>{n}: "You carry something that sings, child."</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>REDCAP, GAKI, BANSHEE, BARGHEST, TROLL, GHOUL, ONI, KAPPA, LAMIA, WRAITH, IMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>folklore</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Remarks on a NOTICED aura</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>{n}: "I smelled you two rooms away."</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>REDCAP, GAKI, BANSHEE, BARGHEST, TROLL, GHOUL, ONI, KAPPA, LAMIA, WRAITH, IMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>folklore</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Remarks on a LOUD aura</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>{n}: "What have you brought down here, child? It is LOUD."</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>REDCAP, GAKI, BANSHEE, BARGHEST, TROLL, GHOUL, ONI, KAPPA, LAMIA, WRAITH, IMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>folklore</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Remarks on a LOUD aura</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>{n}: "The whole hall can hear your pockets."</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>REDCAP, GAKI, BANSHEE, BARGHEST, TROLL, GHOUL, ONI, KAPPA, LAMIA, WRAITH, IMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>folklore</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>KURA carries a MOON thing</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>{n}: "You carry moonlight, child. She will want it back."</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
         <is>
           <t>REDCAP, GAKI, BANSHEE, BARGHEST, TROLL, GHOUL, ONI, KAPPA, LAMIA, WRAITH, IMP</t>
         </is>
@@ -15011,7 +15910,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -15066,6 +15965,2667 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>v1.04: alignment display names. Machine things (data, hardware, programs) use SIGNAL / HUM / STATIC; folklore uses KEPT / STRAY / FERAL; hybrids use two words (natural half first). Same LAW / NEUTRAL / CHAOS underneath (Roster 'Aura name').</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>v1.04: KURA's AURA reads are in her own modern voice, the only one in the dungeon: about 80% jokey, 20% plain and dry. The moon is solemn when dim, sassy when bright.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="49" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Kind</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>KURA vibe-checks {n}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>KURA checks {n} out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>KURA cold-reads {n}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>KURA side-eyes {n}. Thoroughly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>KURA clocks {n}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>KURA reads {n} like a group chat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>KURA scans {n} head to toe. Judging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>KURA gives {n} a once-over.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>KURA lowkey stares at {n}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>KURA looks at {n} for a long moment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>KURA goes quiet and takes {n} in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Loudness: QUIET</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>It's giving nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Loudness: QUIET</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Barely there. NPC energy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Loudness: QUIET</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Lowkey. Very lowkey.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Loudness: QUIET</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Faint. Like it forgot to have one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Loudness: NOTICED</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>It's giving something.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Loudness: NOTICED</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Okay, it has a vibe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Loudness: NOTICED</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Not loud, but present.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Loudness: NOTICED</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>There, if you look for it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Loudness: LOUD</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Main character energy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Loudness: LOUD</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Way too much aura. Yikes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Loudness: LOUD</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>The aura is aura-ing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Loudness: LOUD</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>It's loud. Like, LOUD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Loudness: LOUD</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Loud enough that the walls noticed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Hint: GRUFF</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>{n} looks basic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Hint: GRUFF</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>{n}'s tastes aren't very refined.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Hint: GRUFF</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Looks like {n} only shops at Wal-Mart.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Hint: GRUFF</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>{n} thinks a rock is a gift. It might be right.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Hint: GRUFF</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>{n} likes things it can throw.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Hint: HAUGHTY</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>{n} only accepts designer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Hint: HAUGHTY</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Expensive taste, no budget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Hint: HAUGHTY</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>It thinks it's that girl.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Hint: HAUGHTY</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>{n} is giving gatekeeper.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Hint: HAUGHTY</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>{n} expects to be paid. Well.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Hint: SLY</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>{n} is eyeing your bag. Sus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Hint: SLY</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>It's running a side hustle, for sure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Hint: SLY</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Main hobby: finessing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Hint: SLY</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>It has thrift store eyes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Hint: SLY</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>{n} is counting your pockets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Hint: PRIM</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>{n} color-codes its closet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Hint: PRIM</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>It wants everything to match. Everything.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Hint: PRIM</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Very clean girl aesthetic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Hint: PRIM</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>One crooked thing and it's over.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Hint: PRIM</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>{n} likes a matching set.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Hint: DREAMY</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>{n} is not in this dungeon mentally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Hint: DREAMY</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Head empty, only vibes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Hint: DREAMY</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>{n} is on a different timeline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Hint: DREAMY</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>It's thinking about something shiny. Probably.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Hint: DREAMY</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>{n} is watching a spot on the wall.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Hint: ATOM SLASHER</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Nope. Nope nope nope.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Mood</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Situation</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>solemn (dim)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Doesn't answer</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>The moon keeps her own counsel tonight.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>solemn (dim)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Doesn't answer</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>The moon looks down, and says nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>solemn (dim)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Doesn't answer</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>KURA asks. The moon only watches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>sassy (bright)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Doesn't answer</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>The moon is busy. Try again in a quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>sassy (bright)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Doesn't answer</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>The moon saw that. Not mad, just disappointed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>sassy (bright)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Doesn't answer</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>The moon heard you. She's choosing not to answer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>sassy (bright)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Doesn't answer</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>The moon is giving you a look.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>sassy (bright)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Doesn't answer</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>The moon says no. Politely, for once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>sassy (bright)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Doesn't answer</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>The moon has been up all night. Ask tomorrow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>solemn (dim)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Asked twice in a night</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>The moon has said what she will tonight.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>solemn (dim)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Asked twice in a night</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>KURA looks to the moon again. She has nothing more tonight.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>sassy (bright)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Asked twice in a night</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>The moon already answered. She doesn't do encores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>sassy (bright)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Asked twice in a night</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Once a night, KURA. She has other people.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>sassy (bright)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Asked twice in a night</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>The moon left you on read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>sassy (bright)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Asked twice in a night</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>The moon has been here four billion years. You got your one question.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>No moon tonight</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>KURA scries the sky... No moon tonight. No one to ask.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>No moon tonight</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>KURA scries the sky... Only the dark, a long way up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Phases: new, wax cresc, wane cresc = solemn; wax gibbous, full, wane gibbous = sassy; the half moons pick either.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Aura strength</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Alignment</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Aura name</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>a bag of loose screws</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>COMMON</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CHAOS</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>STATIC</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>a spent battery</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>COMMON</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>HUM</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>a vending machine coin</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>COMMON</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>LAW</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>a subway token</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>COMMON</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>LAW</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>a burned-out circuit board</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>COMMON</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>STRAY STATIC</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>a neon tube fragment</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>COMMON</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>CHAOS</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>STATIC</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>a tangle of fiber cable</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>COMMON</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>HUM</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>a scratched data disc</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>COMMON</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>LAW</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>an ID card, face scratched</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>COMMON</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>LAW</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>a moth-eaten glove</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>COMMON</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>STRAY</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>a bead of smoky glass</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>COMMON</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>CHAOS</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>a cracked hand mirror</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>COMMON</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>CHAOS</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>a vial of medicine</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>UNCOMMON</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>LAW</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>KEPT</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>a strip of prayer cloth</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>UNCOMMON</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>LAW</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>KEPT</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>a stub of black candle</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>UNCOMMON</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>CHAOS</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>a tin of old matches</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>UNCOMMON</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>STRAY</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>a coil of copper wire</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>UNCOMMON</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>HUM</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>a dead pager</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>UNCOMMON</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>CHAOS</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>STATIC</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>a cracked phone</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>UNCOMMON</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>CHAOS</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>STATIC</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>a cassette with no label</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>UNCOMMON</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>FERAL HUM</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>a VR visor, lens cracked</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>UNCOMMON</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>LAW</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>a rusted iron key</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>UNCOMMON</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>LAW</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>KEPT</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>a bent silver charm</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>UNCOMMON</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>STRAY</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>a page of a burned book</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>UNCOMMON</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>CHAOS</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>a rune scratched into a circuit board</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>RARE</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>STRAY HUM</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>a salt-crusted network cable</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>RARE</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>STRAY HUM</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>a candle stub in a soda can</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>RARE</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>CHAOS</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>FERAL STATIC</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>a charm bracelet of old keycards</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>RARE</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>3</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>LAW</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>a rosary of fiber optic beads</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>RARE</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>3</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>LAW</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>KEPT SIGNAL</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>a sealed jar, humming faintly</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>RARE</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>CHAOS</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>a SIM card in red thread</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>RARE</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>CHAOS</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>FERAL STATIC</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>a graffiti-stained saint's medal</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>RARE</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>STRAY HUM</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>a bullet casing on a leather cord</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>RARE</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>CHAOS</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>a keycard, one corner burned</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>RARE</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>LAW</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>an old COMP chip</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>RARE</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>3</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>LAW</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>a black pearl</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>RARE</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>STRAY</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>a jar of grave salt</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>MYTHIC</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>5</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>LAW</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>KEPT</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>a wax seal, unbroken</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>MYTHIC</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>5</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>LAW</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>KEPT</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>a chipped bone die</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>MYTHIC</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>5</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>CHAOS</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>a sealed reliquary</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>MYTHIC</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>5</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>LAW</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>KEPT</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>a ring of red gold</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>MYTHIC</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>5</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>CHAOS</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>a sword in a rotted sheath</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>MYTHIC</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>5</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>STRAY</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>a moonstone</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>MOON</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>8</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>STRAY</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>a shard of pale moonlight</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>MOON</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>8</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>LAW</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>KEPT</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>a fang still warm</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>MOON</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>8</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>CHAOS</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>a silver-veined horn</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>MOON</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>8</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>CHAOS</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>FERAL</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>spirit</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v1.04.1 and v1.04.2 notes: internal changelog, BEHOLD and line 3 lines in the creature sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ra4YzVt7KpmT8wZQpkPNW
</commit_message>
<xml_diff>
--- a/daily-dungeon-characters.xlsx
+++ b/daily-dungeon-characters.xlsx
@@ -13,9 +13,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personalities" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Omens" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KURA aura reads" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Moon" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Moon" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KURA aura reads" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dungeon" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roster'!$A$1:$F$45</definedName>
@@ -2001,13 +2002,151 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Situation</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Line 3: KURA turns NOTICED</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Something down here turns its head.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Line 3: KURA turns NOTICED</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>The dark takes an interest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Line 3: KURA turns NOTICED</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Somewhere, something sniffs the air.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Line 3: KURA turns LOUD</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>The walls lean in a little.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Line 3: KURA turns LOUD</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>The whole level knows you're here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Line 3: KURA turns LOUD</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Every door is listening.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Line 3: KURA gets quieter</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>The dungeon looks away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Line 3: KURA gets quieter</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>The dark loses interest. Rude.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Line 3: KURA gets quieter</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Things go back to ignoring you.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D160"/>
+  <dimension ref="A1:D161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5510,7 +5649,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Good dog energy. Still a hound.</t>
+          <t>CU SITH has good dog energy. Still a hound.</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5671,29 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>It would like you to throw something.</t>
+          <t>CU SITH would like you to throw something.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>CU SITH</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Party member</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Wants what KURA holds up</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>CU SITH stares at it, then at KURA. Give it?</t>
         </is>
       </c>
     </row>
@@ -5548,7 +5709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E348"/>
+  <dimension ref="A1:E360"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14949,6 +15110,330 @@
         </is>
       </c>
       <c r="E348" t="inlineStr">
+        <is>
+          <t>REDCAP, GAKI, BANSHEE, BARGHEST, TROLL, GHOUL, ONI, KAPPA, LAMIA, WRAITH, IMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Wants what KURA holds up (BEHOLD)</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>{n}: "THAT OBJECT. TRANSFER IT?"</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>PING, DAEMON, CRON, NULL, PACKET, WORM, TRACER</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Wants what KURA holds up (BEHOLD)</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>{n}: "REQUEST: THAT. YES / NO?"</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>PING, DAEMON, CRON, NULL, PACKET, WORM, TRACER</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Wants what KURA holds up (BEHOLD)</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>{n}: "ASSET DETECTED. HAND OVER?"</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>PING, DAEMON, CRON, NULL, PACKET, WORM, TRACER</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>hardware</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Wants what KURA holds up (BEHOLD)</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>{n}: "can I have that? please?"</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>STATIC RAT, PAGER GHOUL, VENDOR, SCRAPPER, DEADLINK, LOOP SHADE</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>hardware</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Wants what KURA holds up (BEHOLD)</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>{n}: "oh. is that for me?"</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>STATIC RAT, PAGER GHOUL, VENDOR, SCRAPPER, DEADLINK, LOOP SHADE</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>hardware</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Wants what KURA holds up (BEHOLD)</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>{n}: "give it here? I'll be careful"</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>STATIC RAT, PAGER GHOUL, VENDOR, SCRAPPER, DEADLINK, LOOP SHADE</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Wants what KURA holds up (BEHOLD)</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>{n}: "That has a pulse. Give it to me?"</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>CHROME HOUND, WIRE WITCH, HEX DRONE, SERVER GOLEM, NEON DRYAD, COIN WRAITH, CHROME ONI, KITSUNE.EXE, PIXEL SPRITE, STATIC BANSHEE, LOOP LICH</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Wants what KURA holds up (BEHOLD)</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>{n}: "I'll take that, traveler. Yes?"</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>CHROME HOUND, WIRE WITCH, HEX DRONE, SERVER GOLEM, NEON DRYAD, COIN WRAITH, CHROME ONI, KITSUNE.EXE, PIXEL SPRITE, STATIC BANSHEE, LOOP LICH</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Wants what KURA holds up (BEHOLD)</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>{n}: "Hand it over, and we're square."</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>CHROME HOUND, WIRE WITCH, HEX DRONE, SERVER GOLEM, NEON DRYAD, COIN WRAITH, CHROME ONI, KITSUNE.EXE, PIXEL SPRITE, STATIC BANSHEE, LOOP LICH</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>folklore</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Wants what KURA holds up (BEHOLD)</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>{n}: "Give it here, child."</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>REDCAP, GAKI, BANSHEE, BARGHEST, TROLL, GHOUL, ONI, KAPPA, LAMIA, WRAITH, IMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>folklore</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Wants what KURA holds up (BEHOLD)</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>{n}: "That. I want that. Well?"</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>REDCAP, GAKI, BANSHEE, BARGHEST, TROLL, GHOUL, ONI, KAPPA, LAMIA, WRAITH, IMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>folklore</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Wants what KURA holds up (BEHOLD)</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>{n}: "A fair thing. Is it mine?"</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
         <is>
           <t>REDCAP, GAKI, BANSHEE, BARGHEST, TROLL, GHOUL, ONI, KAPPA, LAMIA, WRAITH, IMP</t>
         </is>
@@ -15990,23 +16475,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="49" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Part</t>
+          <t>Mood</t>
         </is>
       </c>
       <c r="B1" s="7" t="inlineStr">
         <is>
-          <t>Kind</t>
+          <t>Situation</t>
         </is>
       </c>
       <c r="C1" s="7" t="inlineStr">
@@ -16018,850 +16503,750 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>What KURA does</t>
+          <t>solemn (dim)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Doesn't answer</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>KURA vibe-checks {n}.</t>
+          <t>The moon keeps her own counsel tonight.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>What KURA does</t>
+          <t>solemn (dim)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Doesn't answer</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>KURA checks {n} out.</t>
+          <t>The moon looks down, and says nothing.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>What KURA does</t>
+          <t>solemn (dim)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Doesn't answer</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>KURA cold-reads {n}.</t>
+          <t>KURA asks. The moon only watches.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>What KURA does</t>
+          <t>sassy (bright)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Doesn't answer</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>KURA side-eyes {n}. Thoroughly.</t>
+          <t>The moon is busy. Try again in a quarter.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>What KURA does</t>
+          <t>sassy (bright)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Doesn't answer</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>KURA clocks {n}.</t>
+          <t>The moon saw that. Not mad, just disappointed.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>What KURA does</t>
+          <t>sassy (bright)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Doesn't answer</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>KURA reads {n} like a group chat.</t>
+          <t>The moon heard you. She's choosing not to answer.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>What KURA does</t>
+          <t>sassy (bright)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Doesn't answer</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>KURA scans {n} head to toe. Judging.</t>
+          <t>The moon is giving you a look.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>What KURA does</t>
+          <t>sassy (bright)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Doesn't answer</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>KURA gives {n} a once-over.</t>
+          <t>The moon says no. Politely, for once.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>What KURA does</t>
+          <t>sassy (bright)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Doesn't answer</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>KURA lowkey stares at {n}.</t>
+          <t>The moon has been up all night. Ask tomorrow.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>What KURA does</t>
+          <t>solemn (dim)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>plain</t>
+          <t>Asked twice in a night</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>KURA looks at {n} for a long moment.</t>
+          <t>The moon has said what she will tonight.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>What KURA does</t>
+          <t>solemn (dim)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>plain</t>
+          <t>Asked twice in a night</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>KURA goes quiet and takes {n} in.</t>
+          <t>KURA looks to the moon again. She has nothing more tonight.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Loudness: QUIET</t>
+          <t>sassy (bright)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Asked twice in a night</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>It's giving nothing.</t>
+          <t>The moon already answered. She doesn't do encores.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Loudness: QUIET</t>
+          <t>sassy (bright)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Asked twice in a night</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Barely there. NPC energy.</t>
+          <t>Once a night, KURA. She has other people.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Loudness: QUIET</t>
+          <t>sassy (bright)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Asked twice in a night</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Lowkey. Very lowkey.</t>
+          <t>The moon left you on read.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Loudness: QUIET</t>
+          <t>sassy (bright)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>plain</t>
+          <t>Asked twice in a night</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Faint. Like it forgot to have one.</t>
+          <t>The moon has been here four billion years. You got your one question.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Loudness: NOTICED</t>
-        </is>
-      </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>No moon tonight</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>It's giving something.</t>
+          <t>KURA scries the sky... No moon tonight. No one to ask.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Loudness: NOTICED</t>
-        </is>
-      </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>No moon tonight</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Okay, it has a vibe.</t>
+          <t>KURA scries the sky... Only the dark, a long way up.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Loudness: NOTICED</t>
-        </is>
-      </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Note</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Not loud, but present.</t>
+          <t>Phases: new, wax cresc, wane cresc = solemn; wax gibbous, full, wane gibbous = sassy; the half moons pick either.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Loudness: NOTICED</t>
+          <t>sassy (bright)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>plain</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>There, if you look for it.</t>
+          <t>She's watching you search that wall. Again.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Loudness: LOUD</t>
+          <t>sassy (bright)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Main character energy.</t>
+          <t>That door looked fine, actually.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Loudness: LOUD</t>
+          <t>sassy (bright)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Way too much aura. Yikes.</t>
+          <t>She has seen better climbs. Not many.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Loudness: LOUD</t>
+          <t>sassy (bright)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>The aura is aura-ing.</t>
+          <t>Somewhere overhead, someone is rooting for you. Quietly. Don't make it weird.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Loudness: LOUD</t>
+          <t>sassy (bright)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>It's loud. Like, LOUD.</t>
+          <t>She noticed you didn't eat today.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Loudness: LOUD</t>
+          <t>sassy (bright)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>plain</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Loud enough that the walls noticed.</t>
+          <t>She would like you to know she's full tonight. Thanks for noticing.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Hint: GRUFF</t>
+          <t>sassy (bright)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>{n} looks basic.</t>
+          <t>Pale light pools at her feet, pretending it isn't watching.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Hint: GRUFF</t>
+          <t>sassy (bright)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>{n}'s tastes aren't very refined.</t>
+          <t>A laugh from very high up. Probably not at you.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Hint: GRUFF</t>
+          <t>sassy (bright)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Looks like {n} only shops at Wal-Mart.</t>
+          <t>She's humming something. It isn't for you.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Hint: GRUFF</t>
+          <t>solemn (dim)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>{n} thinks a rock is a gift. It might be right.</t>
+          <t>Far up, she is thin tonight.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Hint: GRUFF</t>
+          <t>solemn (dim)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>plain</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>{n} likes things it can throw.</t>
+          <t>She is listening. Barely.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Hint: HAUGHTY</t>
+          <t>solemn (dim)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>{n} only accepts designer.</t>
+          <t>A sliver of her, watching from very far away.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Hint: HAUGHTY</t>
+          <t>solemn (dim)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Expensive taste, no budget.</t>
+          <t>She's resting. Keep your voice down.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Hint: HAUGHTY</t>
+          <t>solemn (dim)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>It thinks it's that girl.</t>
+          <t>...climb.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Hint: HAUGHTY</t>
+          <t>solemn (dim)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>{n} is giving gatekeeper.</t>
+          <t>Somewhere above, a little light holds on.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Hint: HAUGHTY</t>
+          <t>no moon</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>plain</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>{n} expects to be paid. Well.</t>
+          <t>No moon tonight. Just the dark, being the dark.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Hint: SLY</t>
+          <t>no moon</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>{n} is eyeing your bag. Sus.</t>
+          <t>The sky is empty. She'll be back.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Hint: SLY</t>
+          <t>when KURA is LOUD</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>It's running a side hustle, for sure.</t>
+          <t>She's very aware of your pockets.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Hint: SLY</t>
+          <t>when KURA is LOUD</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Main hobby: finessing.</t>
+          <t>The moon squints at your bag.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Hint: SLY</t>
+          <t>when KURA is LOUD</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, now and then</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>It has thrift store eyes.</t>
+          <t>Bold of you to carry that under her nose.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Hint: SLY</t>
+          <t>reacts</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>plain</t>
+          <t>Line 3, after: fight</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>{n} is counting your pockets.</t>
+          <t>"Messy," says the light from above.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Hint: PRIM</t>
+          <t>reacts</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, after: fight</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>{n} color-codes its closet.</t>
+          <t>Up above, someone winces.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Hint: PRIM</t>
+          <t>reacts</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, after: search</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>It wants everything to match. Everything.</t>
+          <t>She is getting bored...</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Hint: PRIM</t>
+          <t>reacts</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, after: search</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Very clean girl aesthetic.</t>
+          <t>Somewhere above, a long sigh.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Hint: PRIM</t>
+          <t>reacts</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, after: find</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>One crooked thing and it's over.</t>
+          <t>A luminous voice from above: "Fine. That one was good."</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Hint: PRIM</t>
+          <t>reacts</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>plain</t>
+          <t>Line 3, after: find</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>{n} likes a matching set.</t>
+          <t>She approves. Mildly.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Hint: DREAMY</t>
+          <t>reacts</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>jokey</t>
+          <t>Line 3, after: run</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>{n} is not in this dungeon mentally.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Hint: DREAMY</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>jokey</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Head empty, only vibes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Hint: DREAMY</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>jokey</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>{n} is on a different timeline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Hint: DREAMY</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>jokey</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>It's thinking about something shiny. Probably.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Hint: DREAMY</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>plain</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>{n} is watching a spot on the wall.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Hint: ATOM SLASHER</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>jokey</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Nope. Nope nope nope.</t>
+          <t>Up above, someone saw that. She won't tell.</t>
         </is>
       </c>
     </row>
@@ -16871,333 +17256,6 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Mood</t>
-        </is>
-      </c>
-      <c r="B1" s="7" t="inlineStr">
-        <is>
-          <t>Situation</t>
-        </is>
-      </c>
-      <c r="C1" s="7" t="inlineStr">
-        <is>
-          <t>Line</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>solemn (dim)</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Doesn't answer</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>The moon keeps her own counsel tonight.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>solemn (dim)</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Doesn't answer</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>The moon looks down, and says nothing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>solemn (dim)</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Doesn't answer</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>KURA asks. The moon only watches.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>sassy (bright)</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Doesn't answer</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>The moon is busy. Try again in a quarter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>sassy (bright)</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Doesn't answer</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>The moon saw that. Not mad, just disappointed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>sassy (bright)</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Doesn't answer</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>The moon heard you. She's choosing not to answer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>sassy (bright)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Doesn't answer</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>The moon is giving you a look.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>sassy (bright)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Doesn't answer</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>The moon says no. Politely, for once.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>sassy (bright)</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Doesn't answer</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>The moon has been up all night. Ask tomorrow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>solemn (dim)</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Asked twice in a night</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>The moon has said what she will tonight.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>solemn (dim)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Asked twice in a night</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>KURA looks to the moon again. She has nothing more tonight.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>sassy (bright)</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Asked twice in a night</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>The moon already answered. She doesn't do encores.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>sassy (bright)</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Asked twice in a night</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Once a night, KURA. She has other people.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>sassy (bright)</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Asked twice in a night</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>The moon left you on read.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>sassy (bright)</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Asked twice in a night</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>The moon has been here four billion years. You got your one question.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>No moon tonight</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>KURA scries the sky... No moon tonight. No one to ask.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>No moon tonight</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>KURA scries the sky... Only the dark, a long way up.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Phases: new, wax cresc, wane cresc = solemn; wax gibbous, full, wane gibbous = sassy; the half moons pick either.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18629,4 +18687,1026 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C59"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Kind</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>KURA vibe-checks {n}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>KURA checks {n} out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>KURA cold-reads {n}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>KURA side-eyes {n}. Thoroughly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>KURA clocks {n}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>KURA reads {n} like a group chat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>KURA scans {n} head to toe. Judging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>KURA gives {n} a once-over.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>KURA lowkey stares at {n}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>KURA looks at {n} for a long moment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>What KURA does</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>KURA goes quiet and takes {n} in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Loudness: QUIET (after "{n} reads as NAME.")</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>It's giving nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Loudness: QUIET (after "{n} reads as NAME.")</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Barely there. NPC energy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Loudness: QUIET (after "{n} reads as NAME.")</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Lowkey. Very lowkey.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Loudness: QUIET (after "{n} reads as NAME.")</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Faint. Like it forgot to have one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Loudness: NOTICED (after "{n} reads as NAME.")</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>It's giving something.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Loudness: NOTICED (after "{n} reads as NAME.")</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Okay, it has a vibe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Loudness: NOTICED (after "{n} reads as NAME.")</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Not loud, but present.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Loudness: NOTICED (after "{n} reads as NAME.")</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>There, if you look for it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Loudness: LOUD (after "{n} reads as NAME.")</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Main character energy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Loudness: LOUD (after "{n} reads as NAME.")</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Way too much aura. Yikes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Loudness: LOUD (after "{n} reads as NAME.")</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>The aura is aura-ing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Loudness: LOUD (after "{n} reads as NAME.")</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>It's loud. Like, LOUD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Loudness: LOUD (after "{n} reads as NAME.")</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Loud enough that the walls noticed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Hint: GRUFF</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>{n} looks basic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Hint: GRUFF</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>{n}'s tastes aren't very refined.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Hint: GRUFF</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Looks like {n} only shops at Wal-Mart.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Hint: GRUFF</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>{n} thinks a rock is a gift. It might be right.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Hint: GRUFF</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>{n} likes things it can throw.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Hint: HAUGHTY</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>{n} only accepts designer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Hint: HAUGHTY</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>{n} has expensive taste, no budget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Hint: HAUGHTY</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>{n} thinks it's that girl.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Hint: HAUGHTY</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>{n} is giving gatekeeper.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Hint: HAUGHTY</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>{n} expects to be paid. Well.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Hint: SLY</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>{n} is eyeing your bag. Sus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Hint: SLY</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>{n} is running a side hustle, for sure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Hint: SLY</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>{n}'s main hobby is finessing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Hint: SLY</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>{n} has thrift store eyes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Hint: SLY</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>{n} is counting your pockets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Hint: PRIM</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>{n} color-codes its closet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Hint: PRIM</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>{n} wants everything to match. Everything.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Hint: PRIM</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>{n} is very clean girl aesthetic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Hint: PRIM</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>One crooked thing and {n} is over it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Hint: PRIM</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>{n} likes a matching set.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Hint: DREAMY</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>{n} is not in this dungeon mentally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Hint: DREAMY</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>{n} is head empty, only vibes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Hint: DREAMY</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>{n} is on a different timeline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Hint: DREAMY</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>{n} is thinking about something shiny. Probably.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Hint: DREAMY</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>plain</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>{n} is watching a spot on the wall.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Hint: ATOM SLASHER</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>{n}? Nope. Nope nope nope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Line 3: KURA gets hit</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Ow...</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Line 3: KURA gets hit</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>That hurt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Line 3: KURA gets hit</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Okay. Ow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Line 3: KURA gets hit</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Rude.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Line 3: KURA gets hit</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>That's going to bruise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Line 3: KURA gets hit</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Not the face.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Line 3: KURA gets hit</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Ow ow ow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Line 3: KURA gets hit</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>jokey</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Ugh.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
v1.07 notes: real night sky, two-line fight text, INVOKE changes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019XhEKQiLaBVb6sVXSg6pRq
</commit_message>
<xml_diff>
--- a/daily-dungeon-characters.xlsx
+++ b/daily-dungeon-characters.xlsx
@@ -15985,7 +15985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -16861,6 +16861,30 @@
       <c r="C53" t="inlineStr">
         <is>
           <t>The moon has gone quiet. It's late, even for her.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Looking up, she is below the horizon</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>The moon has set.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Looking up, she is below the horizon</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>The moon hasn't risen yet.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v1.09 notes: detailed changelog, dead-end door reads in the sheet, screenshot
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LUdsAdMxuYd1zzXxVrHFk6
</commit_message>
<xml_diff>
--- a/daily-dungeon-characters.xlsx
+++ b/daily-dungeon-characters.xlsx
@@ -19527,7 +19527,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>"Dead end. I can feel it. Spiritually."</t>
+          <t>"Small vibes, the good kind. Someone saved me a seat."</t>
         </is>
       </c>
     </row>
@@ -19544,7 +19544,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>"Small vibes. Nowhere-to-go small."</t>
+          <t>"It's giving cozy corner. Lowkey a hug of a room."</t>
         </is>
       </c>
     </row>

</xml_diff>